<commit_message>
lab01. inspected requirements (1.1.)
</commit_message>
<xml_diff>
--- a/docs/Lab01/CheckLists/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/CheckLists/Lab01_ReviewReport.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Laptop\e\VVSS\CamiVVSS_ro2025-2026\Labs\CheckListsAll\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\bbu\vvss-project\docs\Lab01\CheckLists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE83867-3721-469D-B0A3-67FDA22FF09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE7E496-1190-496B-83CA-0AF0B69FBDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="47">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -135,6 +135,48 @@
   </si>
   <si>
     <t>Effort to perform tool-based code analysis (hours):</t>
+  </si>
+  <si>
+    <t>R01</t>
+  </si>
+  <si>
+    <t>R04</t>
+  </si>
+  <si>
+    <t>R05</t>
+  </si>
+  <si>
+    <t>R06</t>
+  </si>
+  <si>
+    <t>R07</t>
+  </si>
+  <si>
+    <t>does not specify how you can uniquely identify a product, order or ingredients (numeric id, unique name etc.)</t>
+  </si>
+  <si>
+    <t>what happens if persistence files do not exist on first run?</t>
+  </si>
+  <si>
+    <t>does not specify exactly how the system knows when a day has finished (through a button, scheduler … )</t>
+  </si>
+  <si>
+    <t>does not specify how you can update a product (what fields are required for a product in order to be edited, are there default values if the field is left empty on edit … )</t>
+  </si>
+  <si>
+    <t>does not specify anything about informing the user about errors</t>
+  </si>
+  <si>
+    <t>where should files be saved?</t>
+  </si>
+  <si>
+    <t>does not specify what happens if an order contains more products than available in stock</t>
+  </si>
+  <si>
+    <t>how are data fields separated in the file? (',', ';' ?)</t>
+  </si>
+  <si>
+    <t>0.5 hrs</t>
   </si>
 </sst>
 </file>
@@ -809,85 +851,114 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E10" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E11" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E12" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E13" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="D14" s="1"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E14" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
+      <c r="C15" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="D15" s="1"/>
-      <c r="E15" s="2"/>
+      <c r="E15" s="2" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
+      <c r="C16" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="D16" s="1"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="E16" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="2"/>
+      <c r="C17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="15"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="3">
@@ -957,7 +1028,9 @@
         <v>8</v>
       </c>
       <c r="D27" s="12"/>
-      <c r="E27" s="1"/>
+      <c r="E27" s="1" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Cocrea Alex - Arhitectura
</commit_message>
<xml_diff>
--- a/docs/Lab01/CheckLists/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/CheckLists/Lab01_ReviewReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Laptop\e\VVSS\CamiVVSS_ro2025-2026\Labs\CheckListsAll\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\vvss-project\docs\Lab01\CheckLists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE83867-3721-469D-B0A3-67FDA22FF09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0881C60-91EA-4AD0-9BBD-71B593DEAD4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15375" yWindow="2805" windowWidth="11175" windowHeight="11385" tabRatio="650" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -19,24 +19,11 @@
     <sheet name="Tool-basedCodeAnalysis" sheetId="8" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="44">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -135,19 +122,59 @@
   </si>
   <si>
     <t>Effort to perform tool-based code analysis (hours):</t>
+  </si>
+  <si>
+    <t>A03</t>
+  </si>
+  <si>
+    <t>Diagram_v1.0.pdf</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>A02</t>
+  </si>
+  <si>
+    <t>Product + CategorieBautura/TipBautura (enum). Ele sunt enum, deci nu se pot gestiona CRUD. Solutie: CategorieBautura/TipBautura ca entitati + repo/service. Product le refera.</t>
+  </si>
+  <si>
+    <t>DrinkShopController + liste (productList, retetaList, etc.). Layering neclar. Solutie: separare pe layers, controller doar apeleaza DrinkShopService (DTO/ViewModel), business-ul ramane in Service.</t>
+  </si>
+  <si>
+    <t>Stoc, IngredientReteta, Reteta. Ingredient e String, pot aparea inconsistente/dubluri. Solutie: introducem entitatea Ingredient; Stoc si IngredientReteta refera Ingredient (nu String).</t>
+  </si>
+  <si>
+    <t>Cocrea Alex</t>
+  </si>
+  <si>
+    <t>Cervinschi Mario</t>
+  </si>
+  <si>
+    <t>Costan Alex</t>
+  </si>
+  <si>
+    <t>13.03.2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -326,79 +353,80 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,19 +735,19 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.26953125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="4" width="16.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6"/>
     <col min="9" max="9" width="21" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.90625" style="6"/>
+    <col min="10" max="10" width="14.42578125" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -730,7 +758,7 @@
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>19</v>
       </c>
@@ -745,14 +773,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
@@ -766,7 +794,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
@@ -780,7 +808,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
@@ -788,14 +816,14 @@
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -809,7 +837,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -817,7 +845,7 @@
       <c r="D10" s="1"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -826,7 +854,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
@@ -835,7 +863,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -844,7 +872,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -853,7 +881,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -862,7 +890,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -871,7 +899,7 @@
       <c r="D16" s="1"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -880,7 +908,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -889,7 +917,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -898,7 +926,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -907,7 +935,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -916,7 +944,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -925,7 +953,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -934,7 +962,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -943,7 +971,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -952,7 +980,7 @@
       <c r="D25" s="3"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C27" s="11" t="s">
         <v>8</v>
       </c>
@@ -979,18 +1007,18 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.26953125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="22.08984375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="4" width="16.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6"/>
+    <col min="9" max="9" width="22.140625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1001,7 +1029,7 @@
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>18</v>
       </c>
@@ -1016,14 +1044,18 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I3" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" s="17">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
@@ -1034,10 +1066,14 @@
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I4" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
@@ -1048,25 +1084,33 @@
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I5" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" s="3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
+      <c r="D6" s="22" t="s">
+        <v>40</v>
+      </c>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
+      <c r="D7" s="22" t="s">
+        <v>43</v>
+      </c>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1080,33 +1124,51 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="C10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="C11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="C12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1115,7 +1177,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1124,7 +1186,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1133,7 +1195,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1142,7 +1204,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1151,7 +1213,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1160,7 +1222,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1169,7 +1231,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1178,7 +1240,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1187,7 +1249,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1196,7 +1258,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1205,7 +1267,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1214,7 +1276,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1223,7 +1285,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1232,7 +1294,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C28" s="11" t="s">
         <v>8</v>
       </c>
@@ -1259,19 +1321,19 @@
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.26953125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="26.7265625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6"/>
+    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1282,7 +1344,7 @@
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>17</v>
       </c>
@@ -1297,14 +1359,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
@@ -1318,7 +1380,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
@@ -1332,7 +1394,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
@@ -1340,14 +1402,14 @@
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1361,7 +1423,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1369,7 +1431,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1378,7 +1440,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
@@ -1387,7 +1449,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1396,7 +1458,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1405,7 +1467,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1414,7 +1476,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1423,7 +1485,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1432,7 +1494,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1441,7 +1503,7 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1450,7 +1512,7 @@
       <c r="D19" s="1"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1459,7 +1521,7 @@
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1468,7 +1530,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1477,7 +1539,7 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1486,7 +1548,7 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1495,7 +1557,7 @@
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1504,7 +1566,7 @@
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1513,7 +1575,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1522,7 +1584,7 @@
       <c r="D27" s="2"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1531,7 +1593,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1540,7 +1602,7 @@
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1549,7 +1611,7 @@
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C32" s="11" t="s">
         <v>8</v>
       </c>
@@ -1576,20 +1638,20 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.26953125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.90625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.6328125" style="6" customWidth="1"/>
-    <col min="7" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="26.7265625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="5" max="5" width="23.85546875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="6" customWidth="1"/>
+    <col min="7" max="8" width="8.85546875" style="6"/>
+    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1600,7 +1662,7 @@
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>31</v>
       </c>
@@ -1615,14 +1677,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
@@ -1634,7 +1696,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
@@ -1646,7 +1708,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>1</v>
@@ -1655,7 +1717,7 @@
       <c r="E6" s="22"/>
       <c r="F6" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1672,7 +1734,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1681,7 +1743,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1691,7 +1753,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
@@ -1701,7 +1763,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1711,7 +1773,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1721,7 +1783,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1731,7 +1793,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1741,7 +1803,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1751,7 +1813,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1761,7 +1823,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1771,7 +1833,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1781,7 +1843,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1791,7 +1853,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1801,7 +1863,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1811,7 +1873,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1821,7 +1883,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1831,7 +1893,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1841,7 +1903,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1851,7 +1913,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1861,7 +1923,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1871,7 +1933,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1881,7 +1943,7 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C32" s="34" t="s">
         <v>32</v>
       </c>
@@ -1889,7 +1951,7 @@
       <c r="E32" s="35"/>
       <c r="F32" s="18"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F35" s="21"/>
     </row>
   </sheetData>

</xml_diff>